<commit_message>
Fix xlsx formatting: consistent fills, proper column widths, borders
- All rows now have fill color (GREP=green, TEXT=yellow) including column D
- Column widths adjusted: A=9, B=55, C=16, D=55
- Consolas font for pattern/replacement columns
- Thin borders, header freeze, auto-filter

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial_rules.xlsx
+++ b/editorial_rules.xlsx
@@ -10,7 +10,9 @@
     <sheet name="Автозамены" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Инструкция" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Автозамены'!$A$1:$D$9</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +37,29 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -58,8 +81,26 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -73,11 +114,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="003060A0"/>
+      </left>
+      <right style="thin">
+        <color rgb="003060A0"/>
+      </right>
+      <top style="thin">
+        <color rgb="003060A0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="003060A0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -86,6 +155,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,211 +544,212 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Найти</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Заменить на</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>GREP</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>[«(]?\s*[Тт][Оо][Пп]\s*[-–]?\s*(\d+)\s*[»)]?</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>«Топ-$1»</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>топ 16 → «Топ-16», (Топ-3) → «Топ-3», «ТОП 10» → «Топ-10»</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>ТЕКСТ</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>лига чемпионов</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Лига чемпионов</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>лига чемпионов → Лига чемпионов (название турнира с заглавной)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>ТЕКСТ</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>чемпионат мира</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Чемпионат мира</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>чемпионат мира → Чемпионат мира (название турнира с заглавной)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>ТЕКСТ</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>чемпионат России</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Чемпионат России</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>чемпионат России → Чемпионат России (название турнира с заглавной)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>ТЕКСТ</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>первый канал</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>Первый канал</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>первый канал → Первый канал (название СМИ с заглавной)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>GREP</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>([А-ЯЁA-Z][А-Яа-яЁёA-Za-z]*)\s+([Аа]рен(?:а|ы|е|у|ой))</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>$1-$2</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Ростех Арена → Ростех-Арена, на ВТБ Арене → на ВТБ-Арене (все падежи)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>ТЕКСТ</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>КАМАЗ</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>КамАЗ</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>КАМАЗ → КамАЗ (правильное написание бренда)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>GREP</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>\u00BB(\.{3}|\u2026)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>$1\u00BB</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>хххх»... → хххх...» (многоточие внутрь кавычек)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add «выстрел»/«снаряд» auto-quoting rules for football metaphors
GREP rules wrap all word forms in guillemets:
- выстрел/выстрелил/выстрелом/прострелил/стрелял/простреливая → «...»
- снаряд/снаряда/снарядом/снарядов → «...»
Includes (?<!«)/(?!») guards against double-quoting.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial_rules.xlsx
+++ b/editorial_rules.xlsx
@@ -146,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -175,6 +175,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -541,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -745,6 +748,50 @@
       <c r="D9" s="9" t="inlineStr">
         <is>
           <t>хххх»... → хххх...» (многоточие внутрь кавычек)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>GREP</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>(?&lt;!«)\b([Вв]ыстрел[а-яёА-ЯЁ]*|[Пп]рострел[а-яёА-ЯЁ]*|[Сс]треля[а-яёА-ЯЁ]*)\b(?!»)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>«$1»</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>выстрелил → «выстрелил», стрелял → «стрелял», прострелил → «прострелил» (метафора в кавычки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>GREP</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>(?&lt;!«)\b([Сс]наряд[а-яёА-ЯЁ]*)\b(?!»)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>«$1»</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>снаряд → «снаряд», снарядом → «снарядом» (метафора в кавычки)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add «стандарт» rule, fix word boundaries for punctuation support
- Replace \b with explicit Cyrillic lookbehind/lookahead for reliable
  word boundary detection and correct handling of trailing punctuation
- Add «стандарт» auto-quoting rule (all forms: стандарта, стандартов...)
- Pattern: (?<![«а-яёА-ЯЁ])(word)(?![а-яёА-ЯЁ»]) ensures:
  - no double-quoting if already in «»
  - no matching inside longer words
  - punctuation (.,!?:;) stays outside guillemets

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial_rules.xlsx
+++ b/editorial_rules.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -759,7 +759,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>(?&lt;!«)\b([Вв]ыстрел[а-яёА-ЯЁ]*|[Пп]рострел[а-яёА-ЯЁ]*|[Сс]треля[а-яёА-ЯЁ]*)\b(?!»)</t>
+          <t>(?&lt;![«а-яёА-ЯЁ])([Вв]ыстрел[а-яёА-ЯЁ]*|[Пп]рострел[а-яёА-ЯЁ]*|[Сс]треля[а-яёА-ЯЁ]*)(?![а-яёА-ЯЁ»])</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>(?&lt;!«)\b([Сс]наряд[а-яёА-ЯЁ]*)\b(?!»)</t>
+          <t>(?&lt;![«а-яёА-ЯЁ])([Сс]наряд[а-яёА-ЯЁ]*)(?![а-яёА-ЯЁ»])</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -792,6 +792,28 @@
       <c r="D11" s="9" t="inlineStr">
         <is>
           <t>снаряд → «снаряд», снарядом → «снарядом» (метафора в кавычки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>GREP</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>(?&lt;![«а-яёА-ЯЁ])([Сс]тандарт[а-яёА-ЯЁ]*)(?![а-яёА-ЯЁ»])</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>«$1»</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>стандарт → «стандарт», со стандарта → со «стандарта» (метафора в кавычки)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add «снаряд» exception for sport adjectives
Two-pass approach: rule 1 wraps all снаряд forms in «»,
rule 2 immediately after removes guillemets when preceded by
футбольный/хоккейный/баскетбольный/волейбольный/гандбольный/
теннисный/бейсбольный/спортивный (literal usage, not metaphor).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial_rules.xlsx
+++ b/editorial_rules.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -803,15 +803,37 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
+          <t>((?:[Фф]утбольн|[Хх]оккейн|[Бб]аскетбольн|[Вв]олейбольн|[Гг]андбольн|[Тт]еннисн|[Бб]ейсбольн|[Сс]портивн)[а-яёА-ЯЁ]*)(\s+)«([Сс]наряд[а-яёА-ЯЁ]*)»</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>$1$2$3</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Исключение: футбольный «снаряд» → футбольный снаряд (не метафора, убираем кавычки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>GREP</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
           <t>(?&lt;![«а-яёА-ЯЁ])([Сс]тандарт[а-яёА-ЯЁ]*)(?![а-яёА-ЯЁ»])</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>«$1»</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>стандарт → «стандарт», со стандарта → со «стандарта» (метафора в кавычки)</t>
         </is>

</xml_diff>

<commit_message>
Fix ellipsis rule to only trigger on direct speech
Previously «Спартак»... would be converted to «Спартак...», which
is wrong — ellipsis should only move inside quotes for direct speech,
not for short names/titles.

New pattern requires minimum 3 words (2+ spaces) inside quotes:
- «Спартак»... — not touched (1 word = name)
- «Локомотив Москва»... — not touched (2 words = full name)
- «Я думаю, это правда»... → «Я думаю, это правда...» (direct speech)

Also sync all earlier fixes to xlsx (Топ-X, Арена, Стандарт, Камаз)
so the editor source of truth matches the generated txt.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial_rules.xlsx
+++ b/editorial_rules.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -583,17 +583,17 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>[«(]?\s*[Тт][Оо][Пп]\s*[-–]?\s*(\d+)\s*[»)]?</t>
+          <t>[Тт][Оо][Пп]\s*[-–]?\s*(\d+)</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>«Топ-$1»</t>
+          <t>Топ-$1</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>топ 16 → «Топ-16», (Топ-3) → «Топ-3», «ТОП 10» → «Топ-10»</t>
+          <t>топ 16 → Топ-16, ТОП-3 → Топ-3 (только ядро слова, окружающие кавычки/скобки не трогает)</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>([А-ЯЁA-Z][А-Яа-яЁёA-Za-z]*)\s+([Аа]рен(?:а|ы|е|у|ой))</t>
+          <t>([А-ЯЁA-Z][А-Яа-яЁёA-Za-z]{2,})\s+([Аа]рен(?:а|ы|е|у|ой))</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Ростех Арена → Ростех-Арена, на ВТБ Арене → на ВТБ-Арене (все падежи)</t>
+          <t>Ростех Арена → Ростех-Арена, ВТБ Арена → ВТБ-Арена. Минимум 3 буквы в имени, чтобы не ловить предлоги (На, В)</t>
         </is>
       </c>
     </row>
@@ -737,17 +737,17 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>\u00BB(\.{3}|\u2026)</t>
+          <t>«([^«»]*\s[^«»]*\s[^«»]*)»(\.{3}|…)</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>$1\u00BB</t>
+          <t>«$1$2»</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>хххх»... → хххх...» (многоточие внутрь кавычек)</t>
+          <t>Многоточие внутрь кавычек только для прямой речи (3+ слов). «Спартак»... не трогает, «Я думаю, это правда»... → «Я думаю, это правда...»</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>(?&lt;![«а-яёА-ЯЁ])([Сс]тандарт[а-яёА-ЯЁ]*)(?![а-яёА-ЯЁ»])</t>
+          <t>(?&lt;![«а-яёА-ЯЁ])([Сс]тандарт(?:а|у|ом|е|ы|ов|ам|ами|ах)?)(?![а-яёА-ЯЁ»])</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -835,7 +835,29 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>стандарт → «стандарт», со стандарта → со «стандарта» (метафора в кавычки)</t>
+          <t>стандарт → «стандарт», со стандарта → со «стандарта». Только падежные формы существительного, не ловит «стандартный», «стандартизация»</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ТЕКСТ</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Камаз</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>КамАЗ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Камаз → КамАЗ (дополнительный вариант написания)</t>
         </is>
       </c>
     </row>

</xml_diff>